<commit_message>
Fix two tariff codes in HS summary 28511 after TARIC verification
Verified the CN/TARIC codes against the published nomenclature instead
of padding the 8-digit codes with zeros. Two were wrong:

- 8203 20 90 -> 8203 20 00 (TARIC 8203200000). The 8203 20 10 /
  8203 20 90 split (tweezers / other) was merged into a single
  8203 20 00 in 2011, so the code used was obsolete.
- TARIC for 3920 10 25 was 3920102500, which does not exist. The
  subheading is subdivided at 10 digits into ...05 (use in certain
  aircraft) and ...90 (other), so the correct code is 3920102590.

3923 50 90 / 3923509000 confirmed unchanged.

Also record the nomenclature walk for 3920 10 25 in the notes, and mark
the third-country duty column as indicative pending a TARIC check at
the date of release.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ekcgyx7UdfYvc2xT1zEL41
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Brenntag_28511.xlsx
+++ b/output/HS_Code_Summary_Brenntag_28511.xlsx
@@ -821,7 +821,7 @@
       </c>
       <c r="O16" s="6" t="inlineStr">
         <is>
-          <t>Clo 3. země</t>
+          <t>Clo 3. země (orient.)</t>
         </is>
       </c>
       <c r="P16" s="6" t="inlineStr">
@@ -853,7 +853,7 @@
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>3920102500</t>
+          <t>3920102590</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
@@ -914,7 +914,7 @@
       </c>
       <c r="R17" s="7" t="inlineStr">
         <is>
-          <t>Švýcarský kód 3920.1000 NENÍ platná podpoložka KN – pro dovoz do EU použit KN 3920 10 25. K ověření tarifním týmem: jde o hadicovou (layflat) fólii, nikoli plochý film – alternativy 3923 21 00 (pytle a sáčky) nebo 3917 32 00 (trubky). Bez CBAM, bez antidumpingu.</t>
+          <t>Švýcarský kód 3920.1000 NENÍ platná podpoložka KN – pro dovoz do EU použit KN 3920 10 25, TARIC 3920 1025 90 (podpoložka …05 je vyhrazena pro použití v letadlech). K ověření tarifním týmem: jde o hadicovou (layflat) fólii, nikoli plochý film – alternativy 3923 21 00 (pytle a sáčky) nebo 3917 32 00 (trubky). Bez CBAM, bez antidumpingu.</t>
         </is>
       </c>
     </row>
@@ -1004,17 +1004,17 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>8203 20 90</t>
+          <t>8203 20 00</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>8203209000</t>
+          <t>8203200000</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Kleště (včetně štípacích kleští), kleštičky, pinzety a podobné nástroje – ostatní</t>
+          <t>Kleště (včetně štípacích kleští), kleštičky, pinzety a podobné nástroje</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
@@ -1070,7 +1070,7 @@
       </c>
       <c r="R19" s="7" t="inlineStr">
         <is>
-          <t>Švýcarský kód 8203.2000; v KN je 8203 20 děleno na 8203 20 10 (pinzety) a 8203 20 90 (ostatní) – 8místné dělení OVĚŘIT v TARIC. Předpoklad: pracovní část z obecného kovu (pozn. 1 ke kap. 82). Antidumping na ruční nářadí míří na původ ČLR – zde CH, neuplatní se.</t>
+          <t>Švýcarský kód 8203.2000; v KN je 8203 20 děleno na 8203 20 10 (pinzety) a 8203 20 00 (ostatní) – 8místné dělení OVĚŘIT v TARIC. Předpoklad: pracovní část z obecného kovu (pozn. 1 ke kap. 82). Antidumping na ruční nářadí míří na původ ČLR – zde CH, neuplatní se.</t>
         </is>
       </c>
     </row>
@@ -1182,7 +1182,7 @@
     <row r="35" ht="45" customHeight="1">
       <c r="A35" s="15" t="inlineStr">
         <is>
-          <t>Žádný z kódů 3920 10 25 / 3923 50 90 / 8203 20 90 není v příloze I nařízení (EU) 2023/956 → CBAM se nevztahuje. Antidumpingová opatření jsou vázána na původ; původ zboží je CH → neuplatní se. Pozn. pro budoucí zásilky: příjemce Brenntag Specialties Czech a.s. NENÍ v registru reference/CBAM_receivers_CZ.xlsx.</t>
+          <t>Žádný z kódů 3920 10 25 / 3923 50 90 / 8203 20 00 není v příloze I nařízení (EU) 2023/956 → CBAM se nevztahuje. Antidumpingová opatření jsou vázána na původ; původ zboží je CH → neuplatní se. Pozn. pro budoucí zásilky: příjemce Brenntag Specialties Czech a.s. NENÍ v registru reference/CBAM_receivers_CZ.xlsx.</t>
         </is>
       </c>
     </row>
@@ -1454,7 +1454,7 @@
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>8203 20 90</t>
+          <t>8203 20 00</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
-          <t>Ověřit 8místné dělení 8203 20 10 / 90 v TARIC</t>
+          <t>KN 8203 20 00 – dřívější dělení 10/90 bylo v r. 2011 sloučeno</t>
         </is>
       </c>
     </row>
@@ -1880,7 +1880,7 @@
     <row r="18">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>8203 20 90</t>
+          <t>8203 20 00</t>
         </is>
       </c>
       <c r="B18" s="27" t="n">
@@ -1960,7 +1960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A110"/>
+  <dimension ref="A1:A114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -2078,7 +2078,7 @@
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">     3920 10 25 … 73,60 + 5,82 = 79,42 kg | 3923 50 90 … 18,04 + 1,43 = 19,47 kg | 8203 20 90 … 0,10 + 0,01 = 0,11 kg</t>
+          <t xml:space="preserve">     3920 10 25 … 73,60 + 5,82 = 79,42 kg | 3923 50 90 … 18,04 + 1,43 = 19,47 kg | 8203 20 00 … 0,10 + 0,01 = 0,11 kg</t>
         </is>
       </c>
     </row>
@@ -2424,195 +2424,223 @@
         </is>
       </c>
     </row>
-    <row r="79" ht="30" customHeight="1">
+    <row r="79" ht="15" customHeight="1">
       <c r="A79" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  3920.1000 (CH) → v KN NEEXISTUJE. Pro EU: KN 3920 10 25 (LDPE, měrná hmotnost &lt; 0,94; tl. 80 µm ≤ 0,125 mm; nepotištěná; není stretch).</t>
-        </is>
-      </c>
-    </row>
-    <row r="80" ht="15" customHeight="1">
+          <t xml:space="preserve">  3920.1000 (CH) → v KN NEEXISTUJE. Pro EU: KN 3920 10 25, TARIC 3920 1025 90.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="30" customHeight="1">
       <c r="A80" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  3923.5090 (CH) → KN 3923 50 90 – shodné.</t>
+          <t xml:space="preserve">     Cesta nomenklaturou: 3920 10 (polymery ethylenu) → tl. nepřesahující 0,125 mm (80 µm) → měrná hmotnost &lt; 0,94 (LDPE)</t>
         </is>
       </c>
     </row>
     <row r="81" ht="30" customHeight="1">
       <c r="A81" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  8203.2000 (CH) → v KN je 8203 20 dále děleno; pro kleštový nástroj 8203 20 90 (8203 20 10 = pinzety). OVĚŘIT V TARIC.</t>
+          <t xml:space="preserve">     → není fólie 20–40 µm pro fotorezist (3920 10 23), není stretch fólie (3920 10 24) → zbytková položka 3920 10 25 „ostatní“</t>
         </is>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1">
       <c r="A82" s="15" t="inlineStr">
         <is>
+          <t xml:space="preserve">     → TARIC: …05 = pro použití v letadlech, …90 = ostatní → 3920 1025 90.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="15" customHeight="1">
+      <c r="A83" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  3923.5090 (CH) → KN 3923 50 90 – shodné.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="30" customHeight="1">
+      <c r="A84" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  8203.2000 (CH) → KN 8203 20 00, TARIC 8203 2000 00. Dřívější dělení 8203 20 10 (pinzety) / 8203 20 90 (ostatní)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="15" customHeight="1">
+      <c r="A85" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     bylo v roce 2011 SLOUČENO do jediné podpoložky 8203 20 00 – tyto staré kódy se již nepoužívají.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="15" customHeight="1">
+      <c r="A86" s="15" t="inlineStr">
+        <is>
           <t>→ Do JSD uvádět kódy KN/TARIC z listu „HS Summary“, NIKOLI kódy z faktury.</t>
         </is>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" s="32">
+    <row r="88">
+      <c r="A88" s="32">
         <f>== POCHYBNOST K ZAŘAZENÍ LINERUNITŮ (pos. 1+2) – KONZULTOVAT TARIFNÍ TÝM ===</f>
         <v/>
       </c>
     </row>
-    <row r="85" ht="30" customHeight="1">
-      <c r="A85" s="15" t="inlineStr">
+    <row r="89" ht="30" customHeight="1">
+      <c r="A89" s="15" t="inlineStr">
         <is>
           <t>Zboží je HADICOVÁ (layflat) fólie z LDPE, nikoli plochý film. Na úrovni 6 míst se obě strany shodují na 3920.10 a popis</t>
         </is>
       </c>
     </row>
-    <row r="86" ht="30" customHeight="1">
-      <c r="A86" s="15" t="inlineStr">
+    <row r="90" ht="30" customHeight="1">
+      <c r="A90" s="15" t="inlineStr">
         <is>
           <t>na faktuře doslova cituje znění čísla 3920 → jako hlavní varianta použito KN 3920 10 25. V úvahu však přicházejí i:</t>
         </is>
       </c>
     </row>
-    <row r="87" ht="15" customHeight="1">
-      <c r="A87" s="15" t="inlineStr">
+    <row r="91" ht="15" customHeight="1">
+      <c r="A91" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  3923 21 00 (pytle a sáčky z polymerů ethylenu) – pokud by šlo o zhotovený obalový výrobek;</t>
         </is>
       </c>
     </row>
-    <row r="88" ht="30" customHeight="1">
-      <c r="A88" s="15" t="inlineStr">
+    <row r="92" ht="30" customHeight="1">
+      <c r="A92" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  3917 32 00 (trubky) – pozn. 8 ke kap. 39 to však omezuje na výrobky pro vedení plynů/kapalin, což zde neplatí.</t>
         </is>
       </c>
     </row>
-    <row r="89" ht="15" customHeight="1">
-      <c r="A89" s="15" t="inlineStr">
+    <row r="93" ht="15" customHeight="1">
+      <c r="A93" s="15" t="inlineStr">
         <is>
           <t>Hodnota položky 6 330 CHF = většina zásilky → doporučeno potvrzení: customs.tariff@mauriceward.com</t>
         </is>
       </c>
     </row>
-    <row r="91">
-      <c r="A91" s="32">
+    <row r="95">
+      <c r="A95" s="32">
         <f>== CBAM ===</f>
         <v/>
       </c>
     </row>
-    <row r="92" ht="15" customHeight="1">
-      <c r="A92" s="15" t="inlineStr">
-        <is>
-          <t>CBAM se NEVZTAHUJE. Kódy 3920 10 25, 3923 50 90 a 8203 20 90 nejsou v příloze I nařízení (EU) 2023/956</t>
-        </is>
-      </c>
-    </row>
-    <row r="93" ht="30" customHeight="1">
-      <c r="A93" s="15" t="inlineStr">
+    <row r="96" ht="15" customHeight="1">
+      <c r="A96" s="15" t="inlineStr">
+        <is>
+          <t>CBAM se NEVZTAHUJE. Kódy 3920 10 25, 3923 50 90 a 8203 20 00 nejsou v příloze I nařízení (EU) 2023/956</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="30" customHeight="1">
+      <c r="A97" s="15" t="inlineStr">
         <is>
           <t>(cement, elektřina, hnojiva, železo a ocel, hliník, vodík). Plasty ani ruční nářadí kap. 82 nejsou zbožím CBAM.</t>
         </is>
       </c>
     </row>
-    <row r="94" ht="30" customHeight="1">
-      <c r="A94" s="15" t="inlineStr">
+    <row r="98" ht="30" customHeight="1">
+      <c r="A98" s="15" t="inlineStr">
         <is>
           <t>⚠ POZNÁMKA PRO BUDOUCÍ ZÁSILKY: příjemce „Brenntag Specialties Czech a.s.“ (Stachovice 176, CZ-74245 Fulnek) NENÍ</t>
         </is>
       </c>
     </row>
-    <row r="95" ht="30" customHeight="1">
-      <c r="A95" s="15" t="inlineStr">
+    <row r="99" ht="30" customHeight="1">
+      <c r="A99" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   v souboru reference/CBAM_receivers_CZ.xlsx (list List1, 100 záznamů) – prověřeno podle názvu firmy i adresy.</t>
         </is>
       </c>
     </row>
-    <row r="96" ht="30" customHeight="1">
-      <c r="A96" s="15" t="inlineStr">
+    <row r="100" ht="30" customHeight="1">
+      <c r="A100" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Pokud pro něj budeme odbavovat zboží CBAM, je nutné zjistit status (Y128 / Y238 / Y137) a doplnit do registru.</t>
         </is>
       </c>
     </row>
-    <row r="98">
-      <c r="A98" s="32">
+    <row r="102">
+      <c r="A102" s="32">
         <f>== ANTIDUMPING / SLEVA / CELNÍ HODNOTA ===</f>
         <v/>
       </c>
     </row>
-    <row r="99" ht="30" customHeight="1">
-      <c r="A99" s="15" t="inlineStr">
+    <row r="103" ht="30" customHeight="1">
+      <c r="A103" s="15" t="inlineStr">
         <is>
           <t>ANTIDUMPING: neuplatní se. Původ CH; antidumpingová cla na ruční nářadí i plastové fólie míří na jiné původy (zejm. ČLR).</t>
         </is>
       </c>
     </row>
-    <row r="100" ht="30" customHeight="1">
-      <c r="A100" s="15" t="inlineStr">
+    <row r="104" ht="30" customHeight="1">
+      <c r="A104" s="15" t="inlineStr">
         <is>
           <t>SLEVA: v dokladech ŽÁDNÁ – poměrné rozpouštění slevy se neuplatnilo. Rozpouštěn byl pouze náklad na obal (přičtení).</t>
         </is>
       </c>
     </row>
-    <row r="101" ht="30" customHeight="1">
-      <c r="A101" s="15" t="inlineStr">
+    <row r="105" ht="30" customHeight="1">
+      <c r="A105" s="15" t="inlineStr">
         <is>
           <t>Pos. 6 je vzorek zdarma „Value for customs purposes only!!“ (2 ks à 1,00 CHF) – hodnota se do celní hodnoty zahrnuje.</t>
         </is>
       </c>
     </row>
-    <row r="102" ht="15" customHeight="1">
-      <c r="A102" s="15" t="inlineStr">
+    <row r="106" ht="15" customHeight="1">
+      <c r="A106" s="15" t="inlineStr">
         <is>
           <t>CELNÍ HODNOTA (EXW + obal): 7 497,00 CHF. Před podáním JSD doplnit dopravné/pojistné na vnější hranici EU.</t>
         </is>
       </c>
     </row>
-    <row r="104">
-      <c r="A104" s="32">
+    <row r="108">
+      <c r="A108" s="32">
         <f>== CO VYŽÁDAT OD DODAVATELE / CO OVĚŘIT ===</f>
         <v/>
       </c>
     </row>
-    <row r="105" ht="15" customHeight="1">
-      <c r="A105" s="15" t="inlineStr">
-        <is>
-          <t>1) EUR.1 – nejjistější řešení sporu o hodnotový limit preferenčního prohlášení (lze bez ohledu na hodnotu).</t>
-        </is>
-      </c>
-    </row>
-    <row r="106" ht="15" customHeight="1">
-      <c r="A106" s="15" t="inlineStr">
-        <is>
-          <t>2) Skutečná hrubá hmotnost zásilky a hmotnost palety – tára 7,26 kg nesedí na dřevěnou půlpaletu.</t>
-        </is>
-      </c>
-    </row>
-    <row r="107" ht="15" customHeight="1">
-      <c r="A107" s="15" t="inlineStr">
-        <is>
-          <t>3) Materiál palety (dřevo / plast) a zda je VRATNÁ – rozhoduje o VPV 5(b) i o započtení do hrubé hmotnosti.</t>
-        </is>
-      </c>
-    </row>
-    <row r="108" ht="15" customHeight="1">
-      <c r="A108" s="15" t="inlineStr">
-        <is>
-          <t>4) Oprava pos. 7: odstranit „DAP - CZ-74245 Fulnek“, aby doklad uváděl jen EXW Raron.</t>
-        </is>
-      </c>
-    </row>
     <row r="109" ht="15" customHeight="1">
       <c r="A109" s="15" t="inlineStr">
         <is>
-          <t>5) Oprava znění preferenční věty na text přílohy IV úmluvy PEM („...of Switzerland preferential origin.“).</t>
+          <t>1) EUR.1 – nejjistější řešení sporu o hodnotový limit preferenčního prohlášení (lze bez ohledu na hodnotu).</t>
         </is>
       </c>
     </row>
     <row r="110" ht="15" customHeight="1">
       <c r="A110" s="15" t="inlineStr">
         <is>
-          <t>6) Ověřit 8místné dělení 8203 20 v TARIC a potvrdit zařazení linerunitů (3920 10 25) tarifním týmem.</t>
+          <t>2) Skutečná hrubá hmotnost zásilky a hmotnost palety – tára 7,26 kg nesedí na dřevěnou půlpaletu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="15" customHeight="1">
+      <c r="A111" s="15" t="inlineStr">
+        <is>
+          <t>3) Materiál palety (dřevo / plast) a zda je VRATNÁ – rozhoduje o VPV 5(b) i o započtení do hrubé hmotnosti.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="15" customHeight="1">
+      <c r="A112" s="15" t="inlineStr">
+        <is>
+          <t>4) Oprava pos. 7: odstranit „DAP - CZ-74245 Fulnek“, aby doklad uváděl jen EXW Raron.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="15" customHeight="1">
+      <c r="A113" s="15" t="inlineStr">
+        <is>
+          <t>5) Oprava znění preferenční věty na text přílohy IV úmluvy PEM („...of Switzerland preferential origin.“).</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="30" customHeight="1">
+      <c r="A114" s="15" t="inlineStr">
+        <is>
+          <t>6) Potvrdit zařazení linerunitů (3920 10 25) tarifním týmem; sazby cla 3. země ověřit v TARIC k datu propuštění.</t>
         </is>
       </c>
     </row>

</xml_diff>